<commit_message>
fix rings and quadrants
</commit_message>
<xml_diff>
--- a/data/swisscom_bedag_stadt zh.xlsx
+++ b/data/swisscom_bedag_stadt zh.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -434,32 +434,27 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>isNew</t>
+          <t>status</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>description</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>tags</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>tags</t>
+          <t>link</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
           <t>linkName</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>link</t>
         </is>
       </c>
     </row>

</xml_diff>